<commit_message>
Add `retirement_date` field to personnel data and documentation, update lockfile
</commit_message>
<xml_diff>
--- a/data-raw/hrmis_data_dictionary.xlsx
+++ b/data-raw/hrmis_data_dictionary.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://worldbankgroup-my.sharepoint.com/personal/iedochie_worldbank_org/Documents/Documents/GitProjects/govhr/data-raw/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wb559885\OneDrive - WBG\Documents\GitProjects\govhr\data-raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="169" documentId="13_ncr:1_{F2C19B56-FF1C-4A59-81F1-FDCA8E376930}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2EEE5789-D82F-4B3D-9BD4-208CC6EA01D6}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C792C68A-C182-4938-BCF5-7F6D2797C8BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Establishment" sheetId="1" r:id="rId1"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="336" uniqueCount="162">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="342" uniqueCount="165">
   <si>
     <t>character</t>
   </si>
@@ -509,6 +509,15 @@
   </si>
   <si>
     <t>Identifier assigned to each person.</t>
+  </si>
+  <si>
+    <t>retirement_date</t>
+  </si>
+  <si>
+    <t>Date of Retirement, could also be proxied by ref_date of first pension payment</t>
+  </si>
+  <si>
+    <t>Date of Retirement</t>
   </si>
 </sst>
 </file>
@@ -1248,7 +1257,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:F13"/>
+  <dimension ref="A1:F14"/>
   <sheetFormatPr defaultColWidth="37.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="16384" width="37.85546875" style="6"/>
@@ -1511,6 +1520,26 @@
         <v>69</v>
       </c>
       <c r="F13" s="6" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" ht="45" x14ac:dyDescent="0.25">
+      <c r="A14" s="6" t="s">
+        <v>164</v>
+      </c>
+      <c r="B14" s="6" t="s">
+        <v>162</v>
+      </c>
+      <c r="C14" s="6" t="s">
+        <v>163</v>
+      </c>
+      <c r="D14" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="E14" s="6" t="s">
+        <v>69</v>
+      </c>
+      <c r="F14" s="6" t="s">
         <v>128</v>
       </c>
     </row>

</xml_diff>